<commit_message>
Feat: methodologically correct export (ACMG vs CPIC vs GWAS separation)
</commit_message>
<xml_diff>
--- a/GENOMIQ_Review_Export.xlsx
+++ b/GENOMIQ_Review_Export.xlsx
@@ -414,16 +414,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G108"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="53" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -439,25 +440,30 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>rsID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Генотип</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Эффект / Фенотип</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Клинический риск</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>ACMG</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
+        <is>
+          <t>Система оценки</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>Рекомендации</t>
         </is>
@@ -476,25 +482,30 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>rs1800566</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>CC</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Ala/Ala</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>Высокая активность</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Базовый риск</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -513,25 +524,30 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>rs1800566</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>CT</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Ala/Val (гетерозигота)</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>Гетерозигота (Ala/Val)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Умеренный риск окислительного стресса</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -550,25 +566,30 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>rs1800566</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Val/Val (гомозигота)</t>
+          <t>TT (Ser/Ser)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Повышенный риск диабетической нефропатии (при СД1/СД2), риск кардиомиопатии при гемохроматозе</t>
+          <t>Гомозигота</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Высокий риск бензольной гематотоксичности (Moran et al.), риск плохой выживаемости при раке молочной железы (Fagerholm et al.)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -577,35 +598,40 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Группа 1: Детоксикация и антиоксидантная защита</t>
+          <t>Группа 2: Иммунная система и воспаление</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NQO1</t>
+          <t>CRP</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CC (Pro/Pro)</t>
+          <t>rs1205</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Норма</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Базовый риск</t>
+          <t>Гомозигота</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Высокий риск криопирин-ассоциированных синдромов (CAPS)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -614,35 +640,40 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Группа 1: Детоксикация и антиоксидантная защита</t>
+          <t>Группа 2: Иммунная система и воспаление</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NQO1</t>
+          <t>CRP</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CT (Pro/Leu)</t>
+          <t>rs1205</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Гетерозигота</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Умеренный риск оксидативного стресса</t>
+          <t>Низкая продукция СРБ</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Риск замедленной регенерации тканей, риск системного ювенильного артрита</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -651,35 +682,40 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Группа 1: Детоксикация и антиоксидантная защита</t>
+          <t>Группа 2: Иммунная система и воспаление</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NQO1</t>
+          <t>CRP</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TT (Leu/Leu)</t>
+          <t>rs1205</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Гомозигота</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Риск рестеноза in-stent при ИБС, риск катаракты (по мышиным моделям)</t>
+          <t>Гетерозигота</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Умеренный риск сердечно-сосудистых событий, риск кровотечений на варфарине</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -688,35 +724,40 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Группа 1: Детоксикация и антиоксидантная защита</t>
+          <t>Группа 2: Иммунная система и воспаление</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NQO1</t>
+          <t>CRP</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CT (Pro/Ser)</t>
+          <t>rs1205</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>Гетерозигота</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Умеренный риск бензольной гематотоксичности</t>
-        </is>
-      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Умеренный риск аутовоспалительных реакций, лучший ответ на TNF-ингибиторы при РА (rs4612666)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -725,35 +766,40 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Группа 1: Детоксикация и антиоксидантная защита</t>
+          <t>Группа 2: Иммунная система и воспаление</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NQO1</t>
+          <t>CRP</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>TT (Ser/Ser)</t>
+          <t>rs1205</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Гомозигота</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Высокий риск бензольной гематотоксичности (Moran et al.), риск плохой выживаемости при раке молочной железы (Fagerholm et al.)</t>
+          <t>Промежуточная продукция</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Pathogenic / Risk factor</t>
+          <t>Базовый риск</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -772,25 +818,30 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>rs1205</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>GG</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Высокая продукция IL-6</t>
-        </is>
-      </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>Высокая продукция СРБ</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>Умеренный риск воспалительных реакций, риск саркомы Капоши при ВИЧ</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
       <c r="G10" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -809,25 +860,30 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>rs1205</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Промежуточная продукция</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Базовый риск</t>
+          <t>Гомозигота</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Повышенный риск сердечно-сосудистых заболеваний, лучший ответ на розувастатин</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -836,35 +892,40 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Группа 2: Иммунная система и воспаление</t>
+          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CRP</t>
+          <t>FUT2</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>rs601338</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Низкая продукция IL-6</t>
+          <t>CC (Se/Se)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Риск замедленной регенерации тканей, риск системного ювенильного артрита</t>
+          <t>Секретор</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Норма, устойчивость к Norwalk virus</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -873,35 +934,40 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Группа 2: Иммунная система и воспаление</t>
+          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CRP</t>
+          <t>FUT2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>rs601338</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Гетерозигота</t>
+          <t>CT (Se/se)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Умеренный риск аутоиммунных и воспалительных заболеваний, риск септического шока</t>
+          <t>Секретор</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Норма</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -910,35 +976,40 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Группа 2: Иммунная система и воспаление</t>
+          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CRP</t>
+          <t>FUT2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>rs601338</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Гомозигота</t>
+          <t>GG (R/R)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Высокий риск воспаления, астмы, СКВ, мигрени</t>
+          <t>Норма</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Базовый риск</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -947,35 +1018,40 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Группа 2: Иммунная система и воспаление</t>
+          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CRP</t>
+          <t>FUT2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>rs601338</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Гетерозигота</t>
+          <t>TT (se/se)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Умеренный риск сердечно-сосудистых событий, риск кровотечений на варфарине</t>
+          <t>Несекретор</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Устойчивость к норовирусу, риск дефицита B12, риск болезни Крона</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -984,35 +1060,40 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Группа 2: Иммунная система и воспаление</t>
+          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CRP</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>rs4588 / rs7041</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>rs4588 TT + rs7041 GG</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>Гомозигота</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Повышенный риск сердечно-сосудистых заболеваний, лучший ответ на розувастатин</t>
-        </is>
-      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Высокий риск дефицита витамина D, риск остеопороза</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -1021,35 +1102,40 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Группа 2: Иммунная система и воспаление</t>
+          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CRP</t>
+          <t>HFE</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>*07:01 Negative</t>
+          <t>rs1800562 / rs1799945</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Норма</t>
+          <t>C282Y (+/-) + H63D (+/-)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Базовый риск</t>
+          <t>Компаунд-гетерозигота</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Повышенный риск гемохроматоза 1 типа</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -1058,35 +1144,40 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Группа 2: Иммунная система и воспаление</t>
+          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CRP</t>
+          <t>HFE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>*07:01 Positive</t>
+          <t>rs1800562 / rs1799945</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Носительство</t>
+          <t>H63D (+/-)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Высокий риск гепатотоксичности на лапатинибе, риск панкреатита на азатиоприне, сниженный ответ на вакцину от гепатита В</t>
+          <t>Гетерозигота</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Риск гемохроматоза (низкий)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -1100,32 +1191,37 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FUT2</t>
+          <t>MTHFD1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CC (FF)</t>
+          <t>rs2236225</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Норма</t>
+          <t>AA (Q/Q)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Базовый риск</t>
+          <t>Сниженная активность фермента (~20% европейцев)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Повышенный риск токсичности метотрексата, ДНТ у плода (материнский фактор)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>GG (R/R) — норма: Стандартные рекомендации. | Метотрексат (ревматоидный артрит, взрослые): носители A-аллеля — нет связи с ответом на терапию, стандартные рекомендации. | Цисплатин + пеметрексед (мезотелиома): носители AA+AG — снижение общей и безрецидивной выживаемости, требуется более тщательный мониторинг. | Фолиевая кислота (беременность): носители AA — снижение риска гестационного диабета (P=0.031) при приёме 1 мг/сут.</t>
         </is>
       </c>
     </row>
@@ -1137,32 +1233,37 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FUT2</t>
+          <t>MTHFD1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>rs2236225</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Норма</t>
+          <t>AG (R/Q)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Базовый риск</t>
+          <t>Промежуточная активность</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Умеренный риск токсичности метотрексата</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>GG (R/R) — норма: Стандартные рекомендации. | Метотрексат (ревматоидный артрит, взрослые): носители A-аллеля — нет связи с ответом на терапию, стандартные рекомендации. | Цисплатин + пеметрексед (мезотелиома): носители AA+AG — снижение общей и безрецидивной выживаемости, требуется более тщательный мониторинг. | Фолиевая кислота (беременность): носители AA — снижение риска гестационного диабета (P=0.031) при приёме 1 мг/сут.</t>
         </is>
       </c>
     </row>
@@ -1174,30 +1275,35 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FUT2</t>
+          <t>VDR</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CC (Se/Se)</t>
+          <t>rs2228570 / rs1544410</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Секретор</t>
+          <t>CT (Ff)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Норма, устойчивость к Norwalk virus</t>
+          <t>Гетерозигота</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Умеренный риск остеопороза, риск невынашивания</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -1211,30 +1317,35 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FUT2</t>
+          <t>VDR</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CT (Se/se)</t>
+          <t>rs2228570 / rs1544410</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Секретор</t>
+          <t>TT (ff)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Норма</t>
+          <t>Гомозигота</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Высокий риск остеопороза, требуется повышенная доза витамина D</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -1243,516 +1354,586 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FUT2</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>TT (se/se)</t>
+          <t>rs1799963 / rs5896</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Несекретор</t>
+          <t>AA (гомозигота)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Устойчивость к норовирусу, риск дефицита B12, риск болезни Крона</t>
+          <t>Значительное повышение протромбина</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Высокий риск тромбоза</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>GG (норма): Стандартные рекомендации. | Варфарин: носители rs5896 T-аллеля — снижение дозы, мониторинг INR.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>FUT2</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GG (R/R)</t>
+          <t>rs1799963 / rs5896</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Норма</t>
+          <t>GA (гетерозигота)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Базовый риск</t>
+          <t>Повышение протромбина на 30%</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Повышенный риск венозного тромбоза (3x)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>GG (норма): Стандартные рекомендации. | Варфарин: носители rs5896 T-аллеля — снижение дозы, мониторинг INR.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>rs4588 CC + rs7041 TT</t>
+          <t>rs1799963 / rs5896</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Норма</t>
+          <t>GG (дикий)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Нормальный уровень 25(OH)D</t>
+          <t>Нормальный уровень протромбина</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>GG (норма): Стандартные рекомендации. | Варфарин: носители rs5896 T-аллеля — снижение дозы, мониторинг INR.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>rs4588 CT / rs7041 TG</t>
+          <t>rs6025</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Гетерозигота</t>
+          <t>CC (дикий)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Умеренный риск дефицита витамина D</t>
+          <t>Нормальный фактор V, чувствителен к APC</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>CC (норма): Стандартные рекомендации. | Eltrombopag, avatrombopag, lusutrombopag: осторожно, тромботический риск.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>rs4588 TT + rs7041 GG</t>
+          <t>rs6025</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Гомозигота</t>
+          <t>CT (гетерозигота)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Высокий риск дефицита витамина D, риск остеопороза</t>
+          <t>APC-резистентность, риск тромбоза в 7 раз</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Повышенный риск ВТЭ; контрацептивы ПРОТИВОПОКАЗАНЫ</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>CC (норма): Стандартные рекомендации. | Eltrombopag, avatrombopag, lusutrombopag: осторожно, тромботический риск.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>HFE</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>C282Y (-/-) и H63D (-/-)</t>
+          <t>rs6025</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Норма</t>
+          <t>TT (гомозигота)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Базовый риск</t>
+          <t>Выраженная APC-резистентность</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Высокий риск ВТЭ (40-80x)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>CC (норма): Стандартные рекомендации. | Eltrombopag, avatrombopag, lusutrombopag: осторожно, тромботический риск.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>HFE</t>
+          <t>LPL</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>H63D (+/-)</t>
+          <t>rs328 / rs1801177</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Гетерозигота</t>
+          <t>CC (S/S)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Риск гемохроматоза (низкий)</t>
+          <t>Нормальная активность LPL</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>CC (S/S) — норма: Стандартные рекомендации. | CG / GG (S447X): Протективный вариант — снижение триглицеридов, повышение ЛПВП. Не требует коррекции, благоприятный профиль. | Носители D36N или редких LOF-вариантов: риск семейной хиломикронемии — контроль триглицеридов, диета с низким содержанием жиров, консультация липидолога. | При лечении пегаспаргазой (дети с ОЛЛ): риск гипертриглицеридемии, мониторинг липидов. | Правастатин: носители rs328 GG — повышенный ответ (снижение общего холестерина). | Фенофибрат: носители rs320 GG — сниженный ответ при гипертриглицеридемии, рассмотреть альтернативу. | Пиоглитазон (СД2): носители rs328 CG+GG — сниженный ответ.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>HFE</t>
+          <t>LPL</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>H63D (+/+)</t>
+          <t>rs328 / rs1801177</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Гомозигота</t>
+          <t>CG (S/X)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Умеренный риск гемохроматоза</t>
+          <t>Повышенная активность LPL, снижение ТГ</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Протективный</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>CC (S/S) — норма: Стандартные рекомендации. | CG / GG (S447X): Протективный вариант — снижение триглицеридов, повышение ЛПВП. Не требует коррекции, благоприятный профиль. | Носители D36N или редких LOF-вариантов: риск семейной хиломикронемии — контроль триглицеридов, диета с низким содержанием жиров, консультация липидолога. | При лечении пегаспаргазой (дети с ОЛЛ): риск гипертриглицеридемии, мониторинг липидов. | Правастатин: носители rs328 GG — повышенный ответ (снижение общего холестерина). | Фенофибрат: носители rs320 GG — сниженный ответ при гипертриглицеридемии, рассмотреть альтернативу. | Пиоглитазон (СД2): носители rs328 CG+GG — сниженный ответ.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>HFE</t>
+          <t>LPL</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>C282Y (+/-)</t>
+          <t>rs328 / rs1801177</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Гетерозигота</t>
+          <t>GG (X/X)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Нет риска (при отсутствии второй мутации)</t>
+          <t>Высокая активность LPL</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Протективный (снижение ТГ, повышение ЛПВП)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>CC (S/S) — норма: Стандартные рекомендации. | CG / GG (S447X): Протективный вариант — снижение триглицеридов, повышение ЛПВП. Не требует коррекции, благоприятный профиль. | Носители D36N или редких LOF-вариантов: риск семейной хиломикронемии — контроль триглицеридов, диета с низким содержанием жиров, консультация липидолога. | При лечении пегаспаргазой (дети с ОЛЛ): риск гипертриглицеридемии, мониторинг липидов. | Правастатин: носители rs328 GG — повышенный ответ (снижение общего холестерина). | Фенофибрат: носители rs320 GG — сниженный ответ при гипертриглицеридемии, рассмотреть альтернативу. | Пиоглитазон (СД2): носители rs328 CG+GG — сниженный ответ.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>HFE</t>
+          <t>PCSK9</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>C282Y (+/-) + H63D (+/-)</t>
+          <t>rs11591147 / rs505151</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Компаунд-гетерозигота</t>
+          <t>GG (R/R)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Повышенный риск гемохроматоза 1 типа</t>
+          <t>Нормальная функция PCSK9</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>GG (R/R) — норма: Стандартные рекомендации по контролю LDL-C. | GT / TT (R46L) — протективный: Сниженный риск ИБС, более низкий LDL-C. Не требует коррекции, благоприятный профиль. | Gain-of-function варианты (E670G, редкие): риск семейной гиперхолестеринемии — контроль LDL-C, диета, статины, при недостаточном эффекте — ингибиторы PCSK9 (эволокумаб, алирокумаб, инклисиран). | Статины (аторвастатин и др.): носители rs11591147 T-аллеля — повышенный ответ, 55.6% большее снижение LDL-C. Рассмотреть снижение дозы.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>HFE</t>
+          <t>PCSK9</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>C282Y (+/+)</t>
+          <t>rs11591147 / rs505151</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Гомозигота</t>
+          <t>GT (R/L)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Высокий риск гемохроматоза 1 типа</t>
+          <t>Loss-of-function, снижение PCSK9</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Pathogenic</t>
+          <t>Протективный — снижение LDL-C на 15%, риск ИБС на 47% ниже</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>GG (R/R) — норма: Стандартные рекомендации по контролю LDL-C. | GT / TT (R46L) — протективный: Сниженный риск ИБС, более низкий LDL-C. Не требует коррекции, благоприятный профиль. | Gain-of-function варианты (E670G, редкие): риск семейной гиперхолестеринемии — контроль LDL-C, диета, статины, при недостаточном эффекте — ингибиторы PCSK9 (эволокумаб, алирокумаб, инклисиран). | Статины (аторвастатин и др.): носители rs11591147 T-аллеля — повышенный ответ, 55.6% большее снижение LDL-C. Рассмотреть снижение дозы.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MTHFD1</t>
+          <t>PCSK9</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AG (R/Q)</t>
+          <t>rs11591147 / rs505151</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Промежуточная активность</t>
+          <t>TT (L/L)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Умеренный риск токсичности метотрексата</t>
+          <t>Полная потеря функции</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Протективный — резкое снижение LDL-C</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>GG (R/R) — норма: Стандартные рекомендации. | Метотрексат (ревматоидный артрит, взрослые): носители A-аллеля — нет связи с ответом на терапию, стандартные рекомендации. | Цисплатин + пеметрексед (мезотелиома): носители AA+AG — снижение общей и безрецидивной выживаемости, требуется более тщательный мониторинг. | Фолиевая кислота (беременность): носители AA — снижение риска гестационного диабета (P=0.031) при приёме 1 мг/сут.</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>GG (R/R) — норма: Стандартные рекомендации по контролю LDL-C. | GT / TT (R46L) — протективный: Сниженный риск ИБС, более низкий LDL-C. Не требует коррекции, благоприятный профиль. | Gain-of-function варианты (E670G, редкие): риск семейной гиперхолестеринемии — контроль LDL-C, диета, статины, при недостаточном эффекте — ингибиторы PCSK9 (эволокумаб, алирокумаб, инклисиран). | Статины (аторвастатин и др.): носители rs11591147 T-аллеля — повышенный ответ, 55.6% большее снижение LDL-C. Рассмотреть снижение дозы.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MTHFD1</t>
+          <t>CYP1A2</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AA (Q/Q)</t>
+          <t>rs762551</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Сниженная активность фермента (~20% европейцев)</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Повышенный риск токсичности метотрексата, ДНТ у плода (материнский фактор)</t>
+          <t>Быстрый метаболизатор</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Кофеин быстро выводится. Низкий риск ССЗ. При эпилепсии — повышенный клиренс карбамазепина (риск снижения эффекта)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>GG (R/R) — норма: Стандартные рекомендации. | Метотрексат (ревматоидный артрит, взрослые): носители A-аллеля — нет связи с ответом на терапию, стандартные рекомендации. | Цисплатин + пеметрексед (мезотелиома): носители AA+AG — снижение общей и безрецидивной выживаемости, требуется более тщательный мониторинг. | Фолиевая кислота (беременность): носители AA — снижение риска гестационного диабета (P=0.031) при приёме 1 мг/сут.</t>
+          <t>CPIC / DPWG</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Специфических рекомендаций нет</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>VDR</t>
+          <t>CYP1A2</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CT (Ff)</t>
+          <t>rs762551</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Гетерозигота</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Умеренный риск остеопороза, риск невынашивания</t>
+          <t>Промежуточный метаболизатор</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Умеренный метаболизм кофеина</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
+        <is>
+          <t>CPIC / DPWG</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -1761,35 +1942,40 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>VDR</t>
+          <t>CYP1A2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>TT (ff)</t>
+          <t>rs762551</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Гомозигота</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Высокий риск остеопороза, требуется повышенная доза витамина D</t>
+          <t>Медленный метаболизатор</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Кофеин циркулирует долго. Риск гипертонии и инфаркта при &gt;2-3 чашек в день. Курение ускоряет метаболизм</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
+        <is>
+          <t>CPIC / DPWG</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -1798,553 +1984,616 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>VDR</t>
+          <t>CYP2C19</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>rs4244285 / rs4986893 / rs12248560</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Гетерозигота</t>
+          <t>*2/*2, *2/*3, *3/*3</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Умеренный риск переломов</t>
+          <t>Poor Metabolizer (PM)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Клопидогрел не активируется — замена на тикагрелор/прасугрел. Риск QT на циталопраме. Снижение доз вориконазола, ИПП</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>CPIC / DPWG</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Медленные метаболисты (*2, *3): Лекарство не активируется. Риск повторного инфаркта/тромбоза стента. Рекомендуется замена на тикагрелор или прасугрел. | Быстрые метаболисты: Стандартная доза может быть неэффективна (быстрое вымывание).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Группа 3: Метаболизм витаминов и микроэлементов</t>
+          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>VDR</t>
+          <t>CYP2C9</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>rs1799853 / rs1057910</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Гомозигота</t>
+          <t>*2/*2, *2/*3, *3/*3</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Повышенный риск переломов, лучший ответ на алендронат</t>
+          <t>Poor Metabolizer (PM)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Высокий риск кровотечений на варфарине, фенитоине. ПРОТИВОПОКАЗАН siponimod (*3/*3), deuruxolitinib</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>CPIC / DPWG</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>*1/*2, *1/*3 (Intermediate Metabolizer): Сниженная активность. Требуется осторожное титрование дозы варфарина. | *2/*2, *2/*3, *3/*3 (Poor Metabolizer): Значительное снижение активности. Высокий риск кровотечений на стандартных дозах варфарина и побочных эффектов НПВС (гастропатии).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
+          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>CYP2D6</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>GG (дикий)</t>
+          <t>rs3892097 / rs1065852</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Нормальный уровень протромбина</t>
+          <t>*4/*4, *4/*5, *5/*5, *3/*4</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>Poor Metabolizer (PM)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Высокий риск токсичности для арипипразола, атомоксетина, метопролола. Кодеин не работает. ПРОТИВОПОКАЗАН тиоридазин</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>GG (норма): Стандартные рекомендации. | Варфарин: носители rs5896 T-аллеля — снижение дозы, мониторинг INR.</t>
+          <t>CPIC / DPWG</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Специфических рекомендаций нет</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
+          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>SLCO1B1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GA (гетерозигота)</t>
+          <t>rs4149056</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Повышение протромбина на 30%</t>
+          <t>CC (521 CC)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Повышенный риск венозного тромбоза (3x)</t>
+          <t>Poor function</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Pathogenic / Risk factor</t>
+          <t>Высокий риск миопатии и рабдомиолиза. Максимум 20 мг розувастатина. Альтернатива — правастатин/розувастатин</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>GG (норма): Стандартные рекомендации. | Варфарин: носители rs5896 T-аллеля — снижение дозы, мониторинг INR.</t>
+          <t>CPIC / DPWG</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>TC / CC (Сниженный захват): Концентрация статина в плазме крови повышается в несколько раз. Статины начинают воздействовать на скелетные мышцы. | Рекомендация: Снижение дозы симвастатина или переход на правастатин/розувастатин, которые меньше зависят от этого транспортера.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
+          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>SLCO1B1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>AA (гомозигота)</t>
+          <t>rs4149056</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Значительное повышение протромбина</t>
+          <t>TC (521 TC)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Высокий риск тромбоза</t>
+          <t>Intermediate function</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Pathogenic</t>
+          <t>Повышенный риск миопатии на симвастатине 80 мг. Снижение дозы</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>GG (норма): Стандартные рекомендации. | Варфарин: носители rs5896 T-аллеля — снижение дозы, мониторинг INR.</t>
+          <t>CPIC / DPWG</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>TC / CC (Сниженный захват): Концентрация статина в плазме крови повышается в несколько раз. Статины начинают воздействовать на скелетные мышцы. | Рекомендация: Снижение дозы симвастатина или переход на правастатин/розувастатин, которые меньше зависят от этого транспортера.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
+          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>SLCO1B1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CC (дикий)</t>
+          <t>rs4149056</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Нормальный фактор V, чувствителен к APC</t>
+          <t>TT (521 TT)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>Normal function</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Стандартные дозы</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>CC (норма): Стандартные рекомендации. | Eltrombopag, avatrombopag, lusutrombopag: осторожно, тромботический риск.</t>
+          <t>CPIC / DPWG</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>TC / CC (Сниженный захват): Концентрация статина в плазме крови повышается в несколько раз. Статины начинают воздействовать на скелетные мышцы. | Рекомендация: Снижение дозы симвастатина или переход на правастатин/розувастатин, которые меньше зависят от этого транспортера.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>ACTN3</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CT (гетерозигота)</t>
+          <t>rs1815739</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>APC-резистентность, риск тромбоза в 7 раз</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Повышенный риск ВТЭ; контрацептивы ПРОТИВОПОКАЗАНЫ</t>
+          <t>Нормальный синтез ACTN3. Преобладание или высокая эффективность быстрых мышечных волокон.</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Pathogenic / Risk factor</t>
+          <t>Высокий потенциал в спринте, тяжёлой атлетике, силовых видах спорта.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>CC (норма): Стандартные рекомендации. | Eltrombopag, avatrombopag, lusutrombopag: осторожно, тромботический риск.</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>RR / RX: Ваши мышцы генетически предрасположены к быстрым, мощным сокращениям. Рекомендуются силовые тренировки, кроссфит, короткие дистанции.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>ACTN3</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>TT (гомозигота)</t>
+          <t>rs1815739</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Выраженная APC-резистентность</t>
+          <t>RX</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Высокий риск ВТЭ (40-80x)</t>
+          <t>Сниженный синтез ACTN3. Гетерозигота.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Pathogenic</t>
+          <t>Смешанный тип. Хорошая адаптация к интервальным нагрузкам (футбол, хоккей).</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>CC (норма): Стандартные рекомендации. | Eltrombopag, avatrombopag, lusutrombopag: осторожно, тромботический риск.</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>RR / RX: Ваши мышцы генетически предрасположены к быстрым, мощным сокращениям. Рекомендуются силовые тренировки, кроссфит, короткие дистанции.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>LPL</t>
+          <t>ACTN3</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CC (S/S)</t>
+          <t>rs1815739</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Нормальная активность LPL</t>
+          <t>XX</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>Полное отсутствие белка ACTN3. Компенсация за счёт ACTN2 (медленные волокна).</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Высокий потенциал в видах спорта на выносливость (марафон, плавание на длинные дистанции, велоспорт).</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>CC (S/S) — норма: Стандартные рекомендации. | CG / GG (S447X): Протективный вариант — снижение триглицеридов, повышение ЛПВП. Не требует коррекции, благоприятный профиль. | Носители D36N или редких LOF-вариантов: риск семейной хиломикронемии — контроль триглицеридов, диета с низким содержанием жиров, консультация липидолога. | При лечении пегаспаргазой (дети с ОЛЛ): риск гипертриглицеридемии, мониторинг липидов. | Правастатин: носители rs328 GG — повышенный ответ (снижение общего холестерина). | Фенофибрат: носители rs320 GG — сниженный ответ при гипертриглицеридемии, рассмотреть альтернативу. | Пиоглитазон (СД2): носители rs328 CG+GG — сниженный ответ.</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>RR / RX: Ваши мышцы генетически предрасположены к быстрым, мощным сокращениям. Рекомендуются силовые тренировки, кроссфит, короткие дистанции.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LPL</t>
+          <t>COMT</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CG (S/X)</t>
+          <t>rs4680</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Повышенная активность LPL, снижение ТГ</t>
+          <t>Met/Met</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Протективный</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
+          <t>"Мыслитель" (Worrier)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>CC (S/S) — норма: Стандартные рекомендации. | CG / GG (S447X): Протективный вариант — снижение триглицеридов, повышение ЛПВП. Не требует коррекции, благоприятный профиль. | Носители D36N или редких LOF-вариантов: риск семейной хиломикронемии — контроль триглицеридов, диета с низким содержанием жиров, консультация липидолога. | При лечении пегаспаргазой (дети с ОЛЛ): риск гипертриглицеридемии, мониторинг липидов. | Правастатин: носители rs328 GG — повышенный ответ (снижение общего холестерина). | Фенофибрат: носители rs320 GG — сниженный ответ при гипертриглицеридемии, рассмотреть альтернативу. | Пиоглитазон (СД2): носители rs328 CG+GG — сниженный ответ.</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Специфических рекомендаций нет</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>LPL</t>
+          <t>COMT</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>GG (X/X)</t>
+          <t>rs4680</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Высокая активность LPL</t>
+          <t>Val/Met</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Протективный (снижение ТГ, повышение ЛПВП)</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
+          <t>Смешанный</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>CC (S/S) — норма: Стандартные рекомендации. | CG / GG (S447X): Протективный вариант — снижение триглицеридов, повышение ЛПВП. Не требует коррекции, благоприятный профиль. | Носители D36N или редких LOF-вариантов: риск семейной хиломикронемии — контроль триглицеридов, диета с низким содержанием жиров, консультация липидолога. | При лечении пегаспаргазой (дети с ОЛЛ): риск гипертриглицеридемии, мониторинг липидов. | Правастатин: носители rs328 GG — повышенный ответ (снижение общего холестерина). | Фенофибрат: носители rs320 GG — сниженный ответ при гипертриглицеридемии, рассмотреть альтернативу. | Пиоглитазон (СД2): носители rs328 CG+GG — сниженный ответ.</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Специфических рекомендаций нет</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PCSK9</t>
+          <t>COMT</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>GG (R/R)</t>
+          <t>rs4680</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Нормальная функция PCSK9</t>
+          <t>Val/Val</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Базовый</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
+          <t>"Воин" (Warrior)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>GG (R/R) — норма: Стандартные рекомендации по контролю LDL-C. | GT / TT (R46L) — протективный: Сниженный риск ИБС, более низкий LDL-C. Не требует коррекции, благоприятный профиль. | Gain-of-function варианты (E670G, редкие): риск семейной гиперхолестеринемии — контроль LDL-C, диета, статины, при недостаточном эффекте — ингибиторы PCSK9 (эволокумаб, алирокумаб, инклисиран). | Статины (аторвастатин и др.): носители rs11591147 T-аллеля — повышенный ответ, 55.6% большее снижение LDL-C. Рассмотреть снижение дозы.</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Специфических рекомендаций нет</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PCSK9</t>
+          <t>FTO</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>GT (R/L)</t>
+          <t>rs9939609</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Loss-of-function, снижение PCSK9</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Протективный — снижение LDL-C на 15%, риск ИБС на 47% ниже</t>
+          <t>Сниженный контроль аппетита. Склонность к выбору жирной и сладкой пищи. ИМТ в среднем выше на 1.5-2.0 кг/м². Риск ожирения повышен в 1.7 раз.</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Benign / Protective</t>
+          <t>Повышенный риск ожирения и ассоциированного СД2.</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>GG (R/R) — норма: Стандартные рекомендации по контролю LDL-C. | GT / TT (R46L) — протективный: Сниженный риск ИБС, более низкий LDL-C. Не требует коррекции, благоприятный профиль. | Gain-of-function варианты (E670G, редкие): риск семейной гиперхолестеринемии — контроль LDL-C, диета, статины, при недостаточном эффекте — ингибиторы PCSK9 (эволокумаб, алирокумаб, инклисиран). | Статины (аторвастатин и др.): носители rs11591147 T-аллеля — повышенный ответ, 55.6% большее снижение LDL-C. Рассмотреть снижение дозы.</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Специфических рекомендаций нет</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Группа 4: Липидный обмен и сердечно-сосудистый риск</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PCSK9</t>
+          <t>FTO</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TT (L/L)</t>
+          <t>rs9939609</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Полная потеря функции</t>
+          <t>TA</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Протективный — резкое снижение LDL-C</t>
+          <t>Умеренное нарушение чувства насыщения. ИМТ в среднем на 0.4-1.0 кг/м² выше нормы.</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Benign / Protective</t>
+          <t>Умеренный риск избыточного веса.</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>GG (R/R) — норма: Стандартные рекомендации по контролю LDL-C. | GT / TT (R46L) — протективный: Сниженный риск ИБС, более низкий LDL-C. Не требует коррекции, благоприятный профиль. | Gain-of-function варианты (E670G, редкие): риск семейной гиперхолестеринемии — контроль LDL-C, диета, статины, при недостаточном эффекте — ингибиторы PCSK9 (эволокумаб, алирокумаб, инклисиран). | Статины (аторвастатин и др.): носители rs11591147 T-аллеля — повышенный ответ, 55.6% большее снижение LDL-C. Рассмотреть снижение дозы.</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Специфических рекомендаций нет</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CYP1A2</t>
+          <t>FTO</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>rs9939609</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Быстрый метаболизатор</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Кофеин быстро выводится. Низкий риск ССЗ. При эпилепсии — повышенный клиренс карбамазепина (риск снижения эффекта)</t>
+          <t>Нормальная регуляция аппетита и чувства насыщения.</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Базовый риск ожирения.</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
+        <is>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -2353,35 +2602,40 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CYP1A2</t>
+          <t>MCM6 / LCT</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>rs4988235</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Промежуточный метаболизатор</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Умеренный метаболизм кофеина</t>
+          <t>Первичная гиполактазия. Снижение выработки лактазы у взрослых до 10-20% от уровня младенца.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Риск лактазной недостаточности (вздутие, диарея после молока).</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
+        <is>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -2390,35 +2644,40 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>CYP1A2</t>
+          <t>MCM6 / LCT</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>rs4988235</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Медленный метаболизатор</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Кофеин циркулирует долго. Риск гипертонии и инфаркта при &gt;2-3 чашек в день. Курение ускоряет метаболизм</t>
+          <t>Персистенция лактазы. Выработка фермента сохраняется на достаточном уровне.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Нормальная переносимость лактозы.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
+        <is>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -2427,294 +2686,334 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CYP2C19</t>
+          <t>MCM6 / LCT</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>*1/*1</t>
+          <t>rs4988235</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Normal Metabolizer (NM)</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Стандартные дозы</t>
+          <t>Персистенция лактазы. Высокая активность фермента на протяжении всей жизни.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Нормальная переносимость лактозы.</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Медленные метаболисты (*2, *3): Лекарство не активируется. Риск повторного инфаркта/тромбоза стента. Рекомендуется замена на тикагрелор или прасугрел. | Быстрые метаболисты: Стандартная доза может быть неэффективна (быстрое вымывание).</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Специфических рекомендаций нет</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CYP2C19</t>
+          <t>PPARG</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>*1/*2, *1/*3, *2/*17</t>
+          <t>rs1801282</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Intermediate Metabolizer (IM)</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Клопидогрел — снижение эффекта, риск тромбоза стента. Снижение доз ИПП, циталопрама</t>
+          <t>Базовая, высокая активность рецептора. Способствует накоплению липидов при избытке калорий.</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Базовый (популяционный) риск инсулинорезистентности.</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Медленные метаболисты (*2, *3): Лекарство не активируется. Риск повторного инфаркта/тромбоза стента. Рекомендуется замена на тикагрелор или прасугрел. | Быстрые метаболисты: Стандартная доза может быть неэффективна (быстрое вымывание).</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>CC (Pro/Pro): Требуется контроль простых углеводов и гликемического индекса пищи. Хороший метаболический отклик на добавление Омега-3 ПНЖК в рацион.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CYP2C19</t>
+          <t>PPARG</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>*2/*2, *2/*3, *3/*3</t>
+          <t>rs1801282</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Poor Metabolizer (PM)</t>
+          <t>CG</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Клопидогрел не активируется — замена на тикагрелор/прасугрел. Риск QT на циталопраме. Снижение доз вориконазола, ИПП</t>
+          <t>Сниженная аффинность рецептора. Повышенная чувствительность тканей к инсулину.</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Pathogenic / Risk factor</t>
+          <t>Сниженный (протективный эффект).</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Медленные метаболисты (*2, *3): Лекарство не активируется. Риск повторного инфаркта/тромбоза стента. Рекомендуется замена на тикагрелор или прасугрел. | Быстрые метаболисты: Стандартная доза может быть неэффективна (быстрое вымывание).</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>CC (Pro/Pro): Требуется контроль простых углеводов и гликемического индекса пищи. Хороший метаболический отклик на добавление Омега-3 ПНЖК в рацион.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 6: Нутригенетика и спорт</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>CYP2C19</t>
+          <t>PPARG</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>*1/*17, *17/*17</t>
+          <t>rs1801282</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Rapid / Ultra-rapid Metabolizer (RM/UM)</t>
+          <t>GG</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Риск кровотечений на клопидогреле, ИПП. Снижение эффективности ИПП</t>
+          <t>Значительное улучшение чувствительности к инсулину. Редкий генотип (1-3%).</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Выраженный протективный эффект против СД2.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Медленные метаболисты (*2, *3): Лекарство не активируется. Риск повторного инфаркта/тромбоза стента. Рекомендуется замена на тикагрелор или прасугрел. | Быстрые метаболисты: Стандартная доза может быть неэффективна (быстрое вымывание).</t>
+          <t>GWAS / Evidence-based</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>CC (Pro/Pro): Требуется контроль простых углеводов и гликемического индекса пищи. Хороший метаболический отклик на добавление Омега-3 ПНЖК в рацион.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>CYP2C9</t>
+          <t>MTHFR</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>*1/*1</t>
+          <t>rs1801133 / rs1801131</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Normal Metabolizer (NM)</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Стандартные дозы для всех препаратов</t>
+          <t>Нормальная активность фермента (100%).</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>*1/*2, *1/*3 (Intermediate Metabolizer): Сниженная активность. Требуется осторожное титрование дозы варфарина. | *2/*2, *2/*3, *3/*3 (Poor Metabolizer): Значительное снижение активности. Высокий риск кровотечений на стандартных дозах варфарина и побочных эффектов НПВС (гастропатии).</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>TT или CT+AC: Генетически снижена способность усваивать обычную фолиевую кислоту. Рекомендуется контроль уровня гомоцистеина в крови (целевой уровень обычно &lt; 7-8 мкмоль/л).</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CYP2C9</t>
+          <t>MTHFR</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>*1/*2, *1/*3, *1/*5</t>
+          <t>rs1801133 / rs1801131</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Intermediate Metabolizer (IM)</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Снижение дозы варфарина, фенитоина. Мониторинг INR</t>
+          <t>Снижение активности фермента примерно до 60-65% от нормы.</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Умеренный (при дефиците фолатов)</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>*1/*2, *1/*3 (Intermediate Metabolizer): Сниженная активность. Требуется осторожное титрование дозы варфарина. | *2/*2, *2/*3, *3/*3 (Poor Metabolizer): Значительное снижение активности. Высокий риск кровотечений на стандартных дозах варфарина и побочных эффектов НПВС (гастропатии).</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>TT или CT+AC: Генетически снижена способность усваивать обычную фолиевую кислоту. Рекомендуется контроль уровня гомоцистеина в крови (целевой уровень обычно &lt; 7-8 мкмоль/л).</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>CYP2C9</t>
+          <t>MTHFR</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>*2/*2, *2/*3, *3/*3</t>
+          <t>rs1801133 / rs1801131</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Poor Metabolizer (PM)</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Высокий риск кровотечений на варфарине, фенитоине. ПРОТИВОПОКАЗАН siponimod (*3/*3), deuruxolitinib</t>
+          <t>Выраженное снижение активности (термолабильный вариант, ~30% активности). Значительное повышение уровня гомоцистеина.</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Pathogenic / Risk factor</t>
+          <t>Высокий (ДНТ, невынашивание, ССЗ)</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>*1/*2, *1/*3 (Intermediate Metabolizer): Сниженная активность. Требуется осторожное титрование дозы варфарина. | *2/*2, *2/*3, *3/*3 (Poor Metabolizer): Значительное снижение активности. Высокий риск кровотечений на стандартных дозах варфарина и побочных эффектов НПВС (гастропатии).</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>TT или CT+AC: Генетически снижена способность усваивать обычную фолиевую кислоту. Рекомендуется контроль уровня гомоцистеина в крови (целевой уровень обычно &lt; 7-8 мкмоль/л).</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>CYP2D6</t>
+          <t>MTR</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>*1/*1, *1/*2, *2/*2</t>
+          <t>rs1805087</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Normal Metabolizer (NM)</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Стандартные дозы</t>
+          <t>Нормальная активность метионин-синтазы.</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -2723,35 +3022,40 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CYP2D6</t>
+          <t>MTR</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>*1/*4, *1/*5, *2/*4, *1/*41</t>
+          <t>rs1805087</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Intermediate Metabolizer (IM)</t>
+          <t>AG</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Снижение дозы для тамоксифена, метопролола, антидепрессантов</t>
+          <t>Незначительное снижение ферментативной активности.</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -2760,35 +3064,40 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>CYP2D6</t>
+          <t>MTR</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>*4/*4, *4/*5, *5/*5, *3/*4</t>
+          <t>rs1805087</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Poor Metabolizer (PM)</t>
+          <t>GG</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Высокий риск токсичности для арипипразола, атомоксетина, метопролола. Кодеин не работает. ПРОТИВОПОКАЗАН тиоридазин</t>
+          <t>Снижение активности фермента. Возможна ассоциация с повышением гомоцистеина при недостатке витамина B12.</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Pathogenic / Risk factor</t>
+          <t>Умеренный (зависит от B12)</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -2797,35 +3106,40 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>CYP2D6</t>
+          <t>MTRR</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>*1/*1xN, *1/*2xN</t>
+          <t>rs1801394</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Ultra-rapid Metabolizer (UM)</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ПРОТИВОПОКАЗАН кодеин, трамадол (риск остановки дыхания). Элиглустат не эффективен</t>
+          <t>Нормальное сродство к MTR. Эффективная реактивация метионин-синтазы.</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Pathogenic / Risk factor</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
+        <is>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
         <is>
           <t>Специфических рекомендаций нет</t>
         </is>
@@ -2834,1577 +3148,544 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SLCO1B1</t>
+          <t>MTRR</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>TT (521 TT)</t>
+          <t>rs1801394</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Normal function</t>
+          <t>AG</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Стандартные дозы</t>
+          <t>Сниженная способность реактивировать MTR.</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Низкий/Умеренный</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>TC / CC (Сниженный захват): Концентрация статина в плазме крови повышается в несколько раз. Статины начинают воздействовать на скелетные мышцы. | Рекомендация: Снижение дозы симвастатина или переход на правастатин/розувастатин, которые меньше зависят от этого транспортера.</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Специфических рекомендаций нет</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SLCO1B1</t>
+          <t>MTRR</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>TC (521 TC)</t>
+          <t>rs1801394</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Intermediate function</t>
+          <t>GG</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Повышенный риск миопатии на симвастатине 80 мг. Снижение дозы</t>
+          <t>Значительное снижение эффективности восстановления MTR. В сочетании с дефицитом B12 или мутациями MTHFR ведет к росту гомоцистеина.</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Умеренный (ДНТ)</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>TC / CC (Сниженный захват): Концентрация статина в плазме крови повышается в несколько раз. Статины начинают воздействовать на скелетные мышцы. | Рекомендация: Снижение дозы симвастатина или переход на правастатин/розувастатин, которые меньше зависят от этого транспортера.</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Специфических рекомендаций нет</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Группа 5: Фармакогенетика и метаболизм лекарств</t>
+          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SLCO1B1</t>
+          <t>GSTM1</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>CC (521 CC)</t>
+          <t>rs3754446</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Poor function</t>
+          <t>non-null / null</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Высокий риск миопатии и рабдомиолиза. Максимум 20 мг розувастатина. Альтернатива — правастатин/розувастатин</t>
+          <t>Гетерозиготная делеция</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Pathogenic / Risk factor</t>
+          <t>Умеренный (зависит от препарата)</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>TC / CC (Сниженный захват): Концентрация статина в плазме крови повышается в несколько раз. Статины начинают воздействовать на скелетные мышцы. | Рекомендация: Снижение дозы симвастатина или переход на правастатин/розувастатин, которые меньше зависят от этого транспортера.</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>non-null / non-null (норма): Стандартные рекомендации. | Цисплатин: носители GSTM1 null — повышенный риск ототоксичности и глухоты, особенно при лечении рака яичка. Рекомендуется аудиологический мониторинг. | Бусульфан: носители rs3754446 — изменённый метаболизм, контроль концентрации при ОМЛ.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
+          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ACTN3</t>
+          <t>GSTM1</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>rs3754446</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Нормальный синтез ACTN3. Преобладание или высокая эффективность быстрых мышечных волокон.</t>
+          <t>null / null</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Высокий потенциал в спринте, тяжёлой атлетике, силовых видах спорта.</t>
+          <t>Полная делеция гена</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Высокий риск токсичности при химиотерапии; риск рака лёгкого, мочевого пузыря при курении</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>RR / RX: Ваши мышцы генетически предрасположены к быстрым, мощным сокращениям. Рекомендуются силовые тренировки, кроссфит, короткие дистанции.</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>non-null / non-null (норма): Стандартные рекомендации. | Цисплатин: носители GSTM1 null — повышенный риск ототоксичности и глухоты, особенно при лечении рака яичка. Рекомендуется аудиологический мониторинг. | Бусульфан: носители rs3754446 — изменённый метаболизм, контроль концентрации при ОМЛ.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
+          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ACTN3</t>
+          <t>GSTP1</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>RX</t>
+          <t>rs1695 (A313G)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Сниженный синтез ACTN3. Гетерозигота.</t>
+          <t>AA (Ile/Ile)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Смешанный тип. Хорошая адаптация к интервальным нагрузкам (футбол, хоккей).</t>
+          <t>Нормальная активность фермента</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>RR / RX: Ваши мышцы генетически предрасположены к быстрым, мощным сокращениям. Рекомендуются силовые тренировки, кроссфит, короткие дистанции.</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>AA (норма): Стандартные рекомендации по профилактике онкозаболеваний. | Цисплатин / карбоплатин: носители G-аллеля — изменённый ответ и повышенный риск нейротоксичности, мониторинг.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
+          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ACTN3</t>
+          <t>GSTP1</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>XX</t>
+          <t>rs1695 (A313G)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Полное отсутствие белка ACTN3. Компенсация за счёт ACTN2 (медленные волокна).</t>
+          <t>AG (Ile/Val)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Высокий потенциал в видах спорта на выносливость (марафон, плавание на длинные дистанции, велоспорт).</t>
+          <t>Умеренное снижение активности</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Benign / Trait</t>
+          <t>Умеренный риск рака лёгкого и ротовой полости при курении; изменённая токсичность платиновых препаратов</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>RR / RX: Ваши мышцы генетически предрасположены к быстрым, мощным сокращениям. Рекомендуются силовые тренировки, кроссфит, короткие дистанции.</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>AA (норма): Стандартные рекомендации по профилактике онкозаболеваний. | Цисплатин / карбоплатин: носители G-аллеля — изменённый ответ и повышенный риск нейротоксичности, мониторинг.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
+          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>COMT</t>
+          <t>GSTP1</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Val/Val</t>
+          <t>rs1695 (A313G)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>"Воин" (Warrior)</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr"/>
+          <t>GG (Val/Val)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Выраженное снижение активности</t>
+        </is>
+      </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Высокий риск рака лёгкого, ротовой полости, мочевого пузыря при курении</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>AA (норма): Стандартные рекомендации по профилактике онкозаболеваний. | Цисплатин / карбоплатин: носители G-аллеля — изменённый ответ и повышенный риск нейротоксичности, мониторинг.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
+          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>COMT</t>
+          <t>GSTT1</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Val/Met</t>
+          <t>rs4630</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Смешанный</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr"/>
+          <t>non-null / null</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Гетерозиготная делеция</t>
+        </is>
+      </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Умеренный (зависит от препарата)</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>non-null / non-null (норма): Стандартные рекомендации. | При лечении иматинибом (ХМЛ): носители GSTT1 null могут иметь сниженный ответ, особенно в сочетании с GSTM1 null — обсудить с гематологом. | Иматиниб (ХМЛ): носители GSTT1 null/null — риск неудачи терапии (P=0.021). Особенно высокий риск при сочетании GSTT1 null + GSTM1 null (P&lt;0.001) — рекомендован мониторинг BCR-ABL1.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
+          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>COMT</t>
+          <t>GSTT1</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Met/Met</t>
+          <t>rs4630</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>"Мыслитель" (Worrier)</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr"/>
+          <t>null / null</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Полная делеция гена</t>
+        </is>
+      </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Trait / Normal</t>
+          <t>Снижение эффективности иматиниба при ХМЛ; снижение детоксикации хлорметанов</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>non-null / non-null (норма): Стандартные рекомендации. | При лечении иматинибом (ХМЛ): носители GSTT1 null могут иметь сниженный ответ, особенно в сочетании с GSTM1 null — обсудить с гематологом. | Иматиниб (ХМЛ): носители GSTT1 null/null — риск неудачи терапии (P=0.021). Особенно высокий риск при сочетании GSTT1 null + GSTM1 null (P&lt;0.001) — рекомендован мониторинг BCR-ABL1.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
+          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>FTO</t>
+          <t>NAT2</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>rs1799929 / rs1799930 / rs1799931</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Нормальная регуляция аппетита и чувства насыщения.</t>
+          <t>*5/*5, *6/*6, *5/*6</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Базовый риск ожирения.</t>
+          <t>Slow acetylator</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Benign</t>
+          <t>Высокий (гепатотоксичность изониазида, рак мочевого пузыря)</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>CPIC / DPWG</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Slow / Ultra-slow acetylator: Избегать курения (повышенный риск рака мочевого пузыря и лёгких). При лечении туберкулёза — обязательный контроль функции печени. | Rapid acetylator: Стандартные дозы изониазида могут быть неэффективны — требуется мониторинг концентрации препарата. | Изониазид: Slow acetylators — снижение дозы на 50%; Rapid — повышение до 125% или дважды в день (CPIC 2022). | Гидралазин: Slow acetylators — риск лекарственной волчанки, требуется мониторинг.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
+          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>FTO</t>
+          <t>TP53</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>TA</t>
+          <t>rs1800371 / rs1042522</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Умеренное нарушение чувства насыщения. ИМТ в среднем на 0.4-1.0 кг/м² выше нормы.</t>
+          <t>CC (Pro/Pro)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Умеренный риск избыточного веса.</t>
+          <t>Arg/Arg (по белку)</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>CC (Pro/Pro): Стандартные рекомендации. | CG (Pro/Arg) или GG (Arg/Arg): Регулярные онкоскрининги (лёгкие, желудок, кишечник, грудь). Избегать курения и канцерогенов. Защита от избыточной инсоляции. | Капецитабин / паклитаксел (рак желудка): носители GG (Pro/Pro) — сниженный ответ (P&lt;0.001), обсудить альтернативные схемы. | Препараты платины: носители rs1042522 — влияние на общую выживаемость, мониторинг. | Li-Fraumeni syndrome (патогенные варианты R175H, R248Q, R273H, R282W): наследственный синдром с высоким риском множественных опухолей. Рекомендуется:</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
+          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>FTO</t>
+          <t>TP53</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>rs1800371 / rs1042522</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Сниженный контроль аппетита. Склонность к выбору жирной и сладкой пищи. ИМТ в среднем выше на 1.5-2.0 кг/м². Риск ожирения повышен в 1.7 раз.</t>
+          <t>CG (Pro/Arg)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Повышенный риск ожирения и ассоциированного СД2.</t>
+          <t>Гетерозигота</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Умеренный риск опухолей</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>CC (Pro/Pro): Стандартные рекомендации. | CG (Pro/Arg) или GG (Arg/Arg): Регулярные онкоскрининги (лёгкие, желудок, кишечник, грудь). Избегать курения и канцерогенов. Защита от избыточной инсоляции. | Капецитабин / паклитаксел (рак желудка): носители GG (Pro/Pro) — сниженный ответ (P&lt;0.001), обсудить альтернативные схемы. | Препараты платины: носители rs1042522 — влияние на общую выживаемость, мониторинг. | Li-Fraumeni syndrome (патогенные варианты R175H, R248Q, R273H, R282W): наследственный синдром с высоким риском множественных опухолей. Рекомендуется:</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
+          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MCM6 / LCT</t>
+          <t>TP53</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>rs1800371 / rs1042522</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Первичная гиполактазия. Снижение выработки лактазы у взрослых до 10-20% от уровня младенца.</t>
+          <t>GG (Arg/Arg)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Риск лактазной недостаточности (вздутие, диарея после молока).</t>
+          <t>Pro/Pro (по белку)</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Risk factor</t>
+          <t>Повышенный риск рака лёгких, желудка, колоректального; худший ответ на капецитабин / паклитаксел</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Специфических рекомендаций нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>MCM6 / LCT</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>CT</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Персистенция лактазы. Выработка фермента сохраняется на достаточном уровне.</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Нормальная переносимость лактозы.</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>Специфических рекомендаций нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>MCM6 / LCT</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>TT</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Персистенция лактазы. Высокая активность фермента на протяжении всей жизни.</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Нормальная переносимость лактозы.</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>Специфических рекомендаций нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>PPARG</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Базовая, высокая активность рецептора. Способствует накоплению липидов при избытке калорий.</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Базовый (популяционный) риск инсулинорезистентности.</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>CC (Pro/Pro): Требуется контроль простых углеводов и гликемического индекса пищи. Хороший метаболический отклик на добавление Омега-3 ПНЖК в рацион.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>PPARG</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>CG</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Сниженная аффинность рецептора. Повышенная чувствительность тканей к инсулину.</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>Сниженный (протективный эффект).</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>Likely Benign</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>CC (Pro/Pro): Требуется контроль простых углеводов и гликемического индекса пищи. Хороший метаболический отклик на добавление Омега-3 ПНЖК в рацион.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Группа 6: Нутригенетика и спорт</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>PPARG</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>GG</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Значительное улучшение чувствительности к инсулину. Редкий генотип (1-3%).</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Выраженный протективный эффект против СД2.</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>Likely Benign</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>CC (Pro/Pro): Требуется контроль простых углеводов и гликемического индекса пищи. Хороший метаболический отклик на добавление Омега-3 ПНЖК в рацион.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>MTHFR</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>Нормальная активность фермента (100%).</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Базовый</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>TT или CT+AC: Генетически снижена способность усваивать обычную фолиевую кислоту. Рекомендуется контроль уровня гомоцистеина в крови (целевой уровень обычно &lt; 7-8 мкмоль/л).</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>MTHFR</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>CT</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Снижение активности фермента примерно до 60-65% от нормы.</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Умеренный (при дефиците фолатов)</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>TT или CT+AC: Генетически снижена способность усваивать обычную фолиевую кислоту. Рекомендуется контроль уровня гомоцистеина в крови (целевой уровень обычно &lt; 7-8 мкмоль/л).</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>MTHFR</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>TT</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Выраженное снижение активности (термолабильный вариант, ~30% активности). Значительное повышение уровня гомоцистеина.</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Высокий (ДНТ, невынашивание, ССЗ)</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>Pathogenic / Risk factor</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>TT или CT+AC: Генетически снижена способность усваивать обычную фолиевую кислоту. Рекомендуется контроль уровня гомоцистеина в крови (целевой уровень обычно &lt; 7-8 мкмоль/л).</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>MTR</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>Нормальная активность метионин-синтазы.</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Базовый</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>Специфических рекомендаций нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>MTR</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>AG</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Незначительное снижение ферментативной активности.</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Низкий</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>Likely Benign</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>Специфических рекомендаций нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>MTR</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>GG</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>Снижение активности фермента. Возможна ассоциация с повышением гомоцистеина при недостатке витамина B12.</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Умеренный (зависит от B12)</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>Специфических рекомендаций нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>MTRR</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>Нормальное сродство к MTR. Эффективная реактивация метионин-синтазы.</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Базовый</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>Специфических рекомендаций нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>MTRR</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>AG</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>Сниженная способность реактивировать MTR.</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Низкий/Умеренный</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>Специфических рекомендаций нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>Группа 7: Метаболизм фолатов и метиониновый цикл</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>MTRR</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>GG</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>Значительное снижение эффективности восстановления MTR. В сочетании с дефицитом B12 или мутациями MTHFR ведет к росту гомоцистеина.</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Умеренный (ДНТ)</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>Специфических рекомендаций нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>GSTM1</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>non-null / non-null</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>Нормальная детоксикация</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Базовый</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>non-null / non-null (норма): Стандартные рекомендации. | Цисплатин: носители GSTM1 null — повышенный риск ототоксичности и глухоты, особенно при лечении рака яичка. Рекомендуется аудиологический мониторинг. | Бусульфан: носители rs3754446 — изменённый метаболизм, контроль концентрации при ОМЛ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>GSTM1</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>non-null / null</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>Гетерозиготная делеция</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Умеренный (зависит от препарата)</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>non-null / non-null (норма): Стандартные рекомендации. | Цисплатин: носители GSTM1 null — повышенный риск ототоксичности и глухоты, особенно при лечении рака яичка. Рекомендуется аудиологический мониторинг. | Бусульфан: носители rs3754446 — изменённый метаболизм, контроль концентрации при ОМЛ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>GSTM1</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>null / null</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>Полная делеция гена</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Высокий риск токсичности при химиотерапии; риск рака лёгкого, мочевого пузыря при курении</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>non-null / non-null (норма): Стандартные рекомендации. | Цисплатин: носители GSTM1 null — повышенный риск ототоксичности и глухоты, особенно при лечении рака яичка. Рекомендуется аудиологический мониторинг. | Бусульфан: носители rs3754446 — изменённый метаболизм, контроль концентрации при ОМЛ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>GSTP1</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>AA (Ile/Ile)</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>Нормальная активность фермента</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Базовый</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>AA (норма): Стандартные рекомендации по профилактике онкозаболеваний. | Цисплатин / карбоплатин: носители G-аллеля — изменённый ответ и повышенный риск нейротоксичности, мониторинг.</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>GSTP1</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>AG (Ile/Val)</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>Умеренное снижение активности</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>Умеренный риск рака лёгкого и ротовой полости при курении; изменённая токсичность платиновых препаратов</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>AA (норма): Стандартные рекомендации по профилактике онкозаболеваний. | Цисплатин / карбоплатин: носители G-аллеля — изменённый ответ и повышенный риск нейротоксичности, мониторинг.</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>GSTP1</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>GG (Val/Val)</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>Выраженное снижение активности</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Высокий риск рака лёгкого, ротовой полости, мочевого пузыря при курении</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>AA (норма): Стандартные рекомендации по профилактике онкозаболеваний. | Цисплатин / карбоплатин: носители G-аллеля — изменённый ответ и повышенный риск нейротоксичности, мониторинг.</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>GSTT1</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>non-null / non-null</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>Нормальная детоксикация</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Базовый</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>non-null / non-null (норма): Стандартные рекомендации. | При лечении иматинибом (ХМЛ): носители GSTT1 null могут иметь сниженный ответ, особенно в сочетании с GSTM1 null — обсудить с гематологом. | Иматиниб (ХМЛ): носители GSTT1 null/null — риск неудачи терапии (P=0.021). Особенно высокий риск при сочетании GSTT1 null + GSTM1 null (P&lt;0.001) — рекомендован мониторинг BCR-ABL1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>GSTT1</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>non-null / null</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>Гетерозиготная делеция</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Умеренный (зависит от препарата)</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>non-null / non-null (норма): Стандартные рекомендации. | При лечении иматинибом (ХМЛ): носители GSTT1 null могут иметь сниженный ответ, особенно в сочетании с GSTM1 null — обсудить с гематологом. | Иматиниб (ХМЛ): носители GSTT1 null/null — риск неудачи терапии (P=0.021). Особенно высокий риск при сочетании GSTT1 null + GSTM1 null (P&lt;0.001) — рекомендован мониторинг BCR-ABL1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>GSTT1</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>null / null</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>Полная делеция гена</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>Снижение эффективности иматиниба при ХМЛ; снижение детоксикации хлорметанов</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>non-null / non-null (норма): Стандартные рекомендации. | При лечении иматинибом (ХМЛ): носители GSTT1 null могут иметь сниженный ответ, особенно в сочетании с GSTM1 null — обсудить с гематологом. | Иматиниб (ХМЛ): носители GSTT1 null/null — риск неудачи терапии (P=0.021). Особенно высокий риск при сочетании GSTT1 null + GSTM1 null (P&lt;0.001) — рекомендован мониторинг BCR-ABL1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>NAT2</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>*1/*1, *4/*4</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>Rapid acetylator</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>Базовый</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>Slow / Ultra-slow acetylator: Избегать курения (повышенный риск рака мочевого пузыря и лёгких). При лечении туберкулёза — обязательный контроль функции печени. | Rapid acetylator: Стандартные дозы изониазида могут быть неэффективны — требуется мониторинг концентрации препарата. | Изониазид: Slow acetylators — снижение дозы на 50%; Rapid — повышение до 125% или дважды в день (CPIC 2022). | Гидралазин: Slow acetylators — риск лекарственной волчанки, требуется мониторинг.</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>NAT2</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>*4/*5, *4/*6</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>Intermediate acetylator</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>Умеренный (зависит от препарата)</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>Slow / Ultra-slow acetylator: Избегать курения (повышенный риск рака мочевого пузыря и лёгких). При лечении туберкулёза — обязательный контроль функции печени. | Rapid acetylator: Стандартные дозы изониазида могут быть неэффективны — требуется мониторинг концентрации препарата. | Изониазид: Slow acetylators — снижение дозы на 50%; Rapid — повышение до 125% или дважды в день (CPIC 2022). | Гидралазин: Slow acetylators — риск лекарственной волчанки, требуется мониторинг.</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>NAT2</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>*5/*5, *6/*6, *5/*6</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>Slow acetylator</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>Высокий (гепатотоксичность изониазида, рак мочевого пузыря)</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>Slow / Ultra-slow acetylator: Избегать курения (повышенный риск рака мочевого пузыря и лёгких). При лечении туберкулёза — обязательный контроль функции печени. | Rapid acetylator: Стандартные дозы изониазида могут быть неэффективны — требуется мониторинг концентрации препарата. | Изониазид: Slow acetylators — снижение дозы на 50%; Rapid — повышение до 125% или дважды в день (CPIC 2022). | Гидралазин: Slow acetylators — риск лекарственной волчанки, требуется мониторинг.</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>NAT2</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>*6A/*6A, *6A/*7B, *7B/*7B</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>Ultra-slow acetylator</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>Очень высокий</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>Pathogenic / Risk factor</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>Slow / Ultra-slow acetylator: Избегать курения (повышенный риск рака мочевого пузыря и лёгких). При лечении туберкулёза — обязательный контроль функции печени. | Rapid acetylator: Стандартные дозы изониазида могут быть неэффективны — требуется мониторинг концентрации препарата. | Изониазид: Slow acetylators — снижение дозы на 50%; Rapid — повышение до 125% или дважды в день (CPIC 2022). | Гидралазин: Slow acetylators — риск лекарственной волчанки, требуется мониторинг.</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>TP53</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>CC (Pro/Pro)</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>Arg/Arg (по белку)</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>Базовый</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>Benign</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>CC (Pro/Pro): Стандартные рекомендации. | CG (Pro/Arg) или GG (Arg/Arg): Регулярные онкоскрининги (лёгкие, желудок, кишечник, грудь). Избегать курения и канцерогенов. Защита от избыточной инсоляции. | Капецитабин / паклитаксел (рак желудка): носители GG (Pro/Pro) — сниженный ответ (P&lt;0.001), обсудить альтернативные схемы. | Препараты платины: носители rs1042522 — влияние на общую выживаемость, мониторинг. | Li-Fraumeni syndrome (патогенные варианты R175H, R248Q, R273H, R282W): наследственный синдром с высоким риском множественных опухолей. Рекомендуется:</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>TP53</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>CG (Pro/Arg)</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>Гетерозигота</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>Умеренный риск опухолей</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>Benign / Risk factor</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>CC (Pro/Pro): Стандартные рекомендации. | CG (Pro/Arg) или GG (Arg/Arg): Регулярные онкоскрининги (лёгкие, желудок, кишечник, грудь). Избегать курения и канцерогенов. Защита от избыточной инсоляции. | Капецитабин / паклитаксел (рак желудка): носители GG (Pro/Pro) — сниженный ответ (P&lt;0.001), обсудить альтернативные схемы. | Препараты платины: носители rs1042522 — влияние на общую выживаемость, мониторинг. | Li-Fraumeni syndrome (патогенные варианты R175H, R248Q, R273H, R282W): наследственный синдром с высоким риском множественных опухолей. Рекомендуется:</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>Группа 8: Онкогенетика и метаболизм канцерогенов</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>TP53</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>GG (Arg/Arg)</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>Pro/Pro (по белку)</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Повышенный риск рака лёгких, желудка, колоректального; худший ответ на капецитабин / паклитаксел</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>Risk factor</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
+          <t>ACMG</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
         <is>
           <t>CC (Pro/Pro): Стандартные рекомендации. | CG (Pro/Arg) или GG (Arg/Arg): Регулярные онкоскрининги (лёгкие, желудок, кишечник, грудь). Избегать курения и канцерогенов. Защита от избыточной инсоляции. | Капецитабин / паклитаксел (рак желудка): носители GG (Pro/Pro) — сниженный ответ (P&lt;0.001), обсудить альтернативные схемы. | Препараты платины: носители rs1042522 — влияние на общую выживаемость, мониторинг. | Li-Fraumeni syndrome (патогенные варианты R175H, R248Q, R273H, R282W): наследственный синдром с высоким риском множественных опухолей. Рекомендуется:</t>
         </is>
@@ -4421,10 +3702,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4451,26 +3732,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Что проверять: корректность сопоставления генотипов (колонка 3) с клиническими эффектами и рисками.</t>
+          <t>Что проверять: корректность сопоставления генотипов (колонка 4) с клиническими эффектами и рисками.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Источники: OMIM, ClinVar, PharmGKB, CPIC.</t>
+          <t>Источники: OMIM, ClinVar, PharmGKB, CPIC, FDA, EMA.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Примечание: Колонка 'Рекомендации' содержит только практические выжимки из гайдлайнов.</t>
+          <t>Колонка 'rsID' содержит идентификаторы SNP.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>ВАЖНО: Система оценки разделена методологически. Для моногенных болезней — ACMG. Для фармакогенов — CPIC/DPWG. Для предрасположенностей — GWAS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Контакт: hello@tim-park.online</t>
         </is>

</xml_diff>